<commit_message>
feat: circulo rojo en cuotas, contacto form03, entidad bancaria fija 37.76
</commit_message>
<xml_diff>
--- a/static/parametros_contrato_prenda_v8.xlsx
+++ b/static/parametros_contrato_prenda_v8.xlsx
@@ -2391,25 +2391,25 @@
       </c>
     </row>
     <row r="81" ht="15.75" customHeight="1" s="21">
-      <c r="A81" t="inlineStr">
+      <c r="A81" s="0" t="inlineStr">
         <is>
           <t>37.76</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B81" s="0" t="inlineStr">
         <is>
           <t>habitualista</t>
         </is>
       </c>
-      <c r="C81" t="n">
+      <c r="C81" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D81" s="0" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E81" s="0" t="inlineStr">
         <is>
           <t>x</t>
         </is>
@@ -3360,7 +3360,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E63"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="29.43" customWidth="1" style="21" min="1" max="1"/>
@@ -4767,25 +4767,50 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr">
+      <c r="A62" s="0" t="inlineStr">
         <is>
           <t>38.76</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
+      <c r="B62" s="0" t="inlineStr">
         <is>
           <t>habitualista</t>
         </is>
       </c>
-      <c r="C62" t="n">
+      <c r="C62" s="0" t="n">
         <v>1</v>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="0" t="inlineStr">
         <is>
           <t>Entidad bancaria</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E62" s="0" t="inlineStr">
+        <is>
+          <t>Entidad bancaria</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>37.76</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>entidad bancaria fija h1</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Entidad bancaria</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
         <is>
           <t>Entidad bancaria</t>
         </is>
@@ -4811,7 +4836,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="30.71" customWidth="1" style="21" min="2" max="2"/>
@@ -6573,10 +6598,74 @@
       <c r="F54" s="20" t="n"/>
       <c r="G54" s="20" t="n"/>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>20.32</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>datos contacto supervielle l1</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Entidad Bancaria 01143248000</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Entidad Bancaria 01143248000</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Entidad Bancaria 01143248000</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Entidad Bancaria 01143248000</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>20.34</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>datos contacto supervielle l2</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>prendarios@supervielle.com.ar</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>prendarios@supervielle.com.ar</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>prendarios@supervielle.com.ar</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>prendarios@supervielle.com.ar</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A33:G33"/>
-    <mergeCell ref="A38:G38"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>